<commit_message>
Remove: Extra BOM #29
</commit_message>
<xml_diff>
--- a/Design Files/Balancer-v7.0.2/BOM/Client-BOM-Balancer-v7.0.2.xlsx
+++ b/Design Files/Balancer-v7.0.2/BOM/Client-BOM-Balancer-v7.0.2.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\gerholdvoorde-dronebms\Design Files\Balancer-v7.0.2\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\gerholdvoorde-dronebms\Design Files\Balancer-v7.0.2\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="75">
   <si>
     <t>#</t>
   </si>
@@ -238,9 +238,6 @@
   </si>
   <si>
     <t>-</t>
-  </si>
-  <si>
-    <t>Connector used by client (No part number)</t>
   </si>
   <si>
     <t>DS-B01F-A-7P-S2</t>
@@ -325,7 +322,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -406,21 +403,6 @@
         <color indexed="64"/>
       </left>
       <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
@@ -472,11 +454,11 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -789,9 +771,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -954,7 +936,7 @@
       </c>
       <c r="K6" s="9"/>
     </row>
-    <row r="7" spans="1:11" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="11">
         <f>ROW(B7) - ROW($B$2)</f>
@@ -973,10 +955,10 @@
         <v>34</v>
       </c>
       <c r="G7" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="H7" s="7" t="s">
         <v>74</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>75</v>
       </c>
       <c r="I7" s="8" t="s">
         <v>62</v>
@@ -984,9 +966,7 @@
       <c r="J7" s="7">
         <v>1</v>
       </c>
-      <c r="K7" s="14" t="s">
-        <v>73</v>
-      </c>
+      <c r="K7" s="15"/>
     </row>
     <row r="8" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1148,7 +1128,7 @@
       </c>
       <c r="K12" s="9"/>
     </row>
-    <row r="13" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="11">
         <f>ROW(B13) - ROW($B$2)</f>

</xml_diff>